<commit_message>
Fill in いいかいご office address and phone/fax
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019FEKn7HFzGRhKMsA45fWaY
</commit_message>
<xml_diff>
--- a/output/重要事項説明書_訪問介護_いいかいご.xlsx
+++ b/output/重要事項説明書_訪問介護_いいかいご.xlsx
@@ -77,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -100,10 +100,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -658,20 +654,20 @@
       <c r="D16" s="8" t="n"/>
       <c r="E16" s="8" t="n"/>
     </row>
-    <row r="17" ht="18" customHeight="1">
+    <row r="17" ht="30" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
           <t>事業所所在地</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>【要入力】</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="8" t="n"/>
-      <c r="E17" s="8" t="n"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>〒543-0023 大阪府大阪市天王寺区味原町13-18 オーセント味原302号室</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="n"/>
+      <c r="D17" s="4" t="n"/>
+      <c r="E17" s="4" t="n"/>
     </row>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
@@ -680,16 +676,16 @@
 相談担当者名</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>TEL：【要入力】 FAX：【要入力】
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>TEL：06-4400-9333 FAX：06-4400-9332
 いいかいご事業部
 生田 友哉</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n"/>
-      <c r="D18" s="8" t="n"/>
-      <c r="E18" s="8" t="n"/>
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
+      <c r="E18" s="4" t="n"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
@@ -2821,15 +2817,11 @@
       </c>
     </row>
     <row r="223" ht="18" customHeight="1">
-      <c r="A223" s="10" t="inlineStr">
-        <is>
-          <t>氏名 生田 友哉（連絡先：【要入力】）</t>
-        </is>
-      </c>
-      <c r="B223" s="11" t="n"/>
-      <c r="C223" s="11" t="n"/>
-      <c r="D223" s="11" t="n"/>
-      <c r="E223" s="11" t="n"/>
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>氏名 生田 友哉（連絡先：06-4400-9333）</t>
+        </is>
+      </c>
     </row>
     <row r="224" ht="45" customHeight="1">
       <c r="A224" s="2" t="inlineStr">
@@ -2868,7 +2860,7 @@
         </is>
       </c>
     </row>
-    <row r="230" ht="60" customHeight="1">
+    <row r="230" ht="75" customHeight="1">
       <c r="A230" s="6" t="inlineStr">
         <is>
           <t>【事業者の窓口】
@@ -2878,15 +2870,15 @@
         </is>
       </c>
       <c r="B230" s="9" t="n"/>
-      <c r="C230" s="7" t="inlineStr">
-        <is>
-          <t>所在地　【要入力】
-電話番号・ﾌｧｯｸｽ番号　【要入力】
+      <c r="C230" s="3" t="inlineStr">
+        <is>
+          <t>所在地　〒543-0023 大阪府大阪市天王寺区味原町13-18 オーセント味原302号室
+電話番号 06-4400-9333　ﾌｧｯｸｽ番号 06-4400-9332
 受付時間　午前9時～午後6時</t>
         </is>
       </c>
-      <c r="D230" s="8" t="n"/>
-      <c r="E230" s="8" t="n"/>
+      <c r="D230" s="4" t="n"/>
+      <c r="E230" s="4" t="n"/>
     </row>
     <row r="231" ht="60" customHeight="1">
       <c r="A231" s="6" t="inlineStr">
@@ -3501,96 +3493,96 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="10" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>法人名</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>株式会社AA → 株式会社dhpケアマネジメント（ご指示どおり）</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>事業所名</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>ええかいご → いいかいご（ご指示どおり）</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>管理者・サービス提供責任者等</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>抜屋 壮勇 → 生田 友哉（ご指示どおり）</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>黄色セル</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>【要入力】：いいかいご／新法人の情報が手元にないため空欄。代表者氏名・本社所在地・法人設立年月日・事業所番号・事業所所在地・電話/FAX・苦情窓口所在地など</t>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>【要入力】：いいかいご／新法人の情報が手元にないため空欄。代表者氏名・本社所在地・法人設立年月日・指定事業所番号・署名欄の事業者所在地</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>コメント付きセル</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>旧事業所の内容をそのまま残した箇所（実施地域・損害賠償保険など）。要確認</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>説明年月日・利用者欄</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>新しく使えるよう空欄にしています</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>元の資料</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>重要事項説明書（訪問介護用）写真15ページ（重複1枚を除外）</t>
         </is>

</xml_diff>

<commit_message>
Add いいかいご designated office number
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019FEKn7HFzGRhKMsA45fWaY
</commit_message>
<xml_diff>
--- a/output/重要事項説明書_訪問介護_いいかいご.xlsx
+++ b/output/重要事項説明書_訪問介護_いいかいご.xlsx
@@ -645,14 +645,14 @@
 事業所番号</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>大阪市指定【要入力】</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="8" t="n"/>
-      <c r="E16" s="8" t="n"/>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>大阪市指定２７７１７０２８２２</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="n"/>
+      <c r="E16" s="4" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
@@ -3548,7 +3548,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>【要入力】：いいかいご／新法人の情報が手元にないため空欄。代表者氏名・本社所在地・法人設立年月日・指定事業所番号・署名欄の事業者所在地</t>
+          <t>【要入力】：いいかいご／新法人の情報が手元にないため空欄。代表者氏名・本社所在地・法人設立年月日・署名欄の事業者所在地</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add head office address and incorporation date
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019FEKn7HFzGRhKMsA45fWaY
</commit_message>
<xml_diff>
--- a/output/重要事項説明書_訪問介護_いいかいご.xlsx
+++ b/output/重要事項説明書_訪問介護_いいかいご.xlsx
@@ -41,7 +41,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -51,11 +51,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -77,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -95,18 +90,11 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -571,23 +559,23 @@
       <c r="D9" s="4" t="n"/>
       <c r="E9" s="4" t="n"/>
     </row>
-    <row r="10" ht="45" customHeight="1">
+    <row r="10" ht="60" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
           <t>本社所在地
 （連絡先及び電話番号等）</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>【要入力】
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>〒541-0058 大阪府大阪市中央区南久宝寺町四丁目5番17号 アップウェル船場 2F
 いいかいご
-TEL：【要入力】 FAX：【要入力】</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="n"/>
-      <c r="D10" s="8" t="n"/>
-      <c r="E10" s="8" t="n"/>
+TEL：06-4400-9333 FAX：06-4400-9332</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="4" t="n"/>
+      <c r="E10" s="4" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
@@ -595,14 +583,14 @@
           <t>法人設立年月日</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>【要入力】</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="8" t="n"/>
-      <c r="E11" s="8" t="n"/>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>平成12年6月8日</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="4" t="n"/>
+      <c r="E11" s="4" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -843,8 +831,8 @@
           <t>職務内容</t>
         </is>
       </c>
-      <c r="C35" s="9" t="n"/>
-      <c r="D35" s="9" t="n"/>
+      <c r="C35" s="7" t="n"/>
+      <c r="D35" s="7" t="n"/>
       <c r="E35" s="6" t="inlineStr">
         <is>
           <t>人員数</t>
@@ -962,14 +950,14 @@
           <t>サービス区分と種類</t>
         </is>
       </c>
-      <c r="B43" s="9" t="n"/>
+      <c r="B43" s="7" t="n"/>
       <c r="C43" s="6" t="inlineStr">
         <is>
           <t>サービスの内容</t>
         </is>
       </c>
-      <c r="D43" s="9" t="n"/>
-      <c r="E43" s="9" t="n"/>
+      <c r="D43" s="7" t="n"/>
+      <c r="E43" s="7" t="n"/>
     </row>
     <row r="44" ht="60" customHeight="1">
       <c r="A44" s="6" t="inlineStr">
@@ -977,7 +965,7 @@
           <t>訪問介護計画の作成</t>
         </is>
       </c>
-      <c r="B44" s="9" t="n"/>
+      <c r="B44" s="7" t="n"/>
       <c r="C44" s="3" t="inlineStr">
         <is>
           <t>利用者に係る居宅介護支援事業者が作成した居宅サービス計画（ケアプラン）に基づき、利用者の意向や心身の状況等のアセスメントを行い、援助の目標に応じて具体的なサービス内容を定めた訪問介護計画を作成します。</t>
@@ -1289,7 +1277,7 @@
 通院等のための乗車又は降車の介助</t>
         </is>
       </c>
-      <c r="B60" s="9" t="n"/>
+      <c r="B60" s="7" t="n"/>
       <c r="C60" s="3" t="inlineStr">
         <is>
           <t>通院等に際して、訪問介護員等が運転する自動車への移動・移乗の介助を行います。（移送に係る運賃は別途必要になります。）</t>
@@ -1553,13 +1541,13 @@
           <t>20分以上45分未満（単位数179）</t>
         </is>
       </c>
-      <c r="C84" s="9" t="n"/>
+      <c r="C84" s="7" t="n"/>
       <c r="D84" s="6" t="inlineStr">
         <is>
           <t>45分以上（単位数220）</t>
         </is>
       </c>
-      <c r="E84" s="9" t="n"/>
+      <c r="E84" s="7" t="n"/>
     </row>
     <row r="85" ht="30" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
@@ -1704,7 +1692,7 @@
           <t>加算</t>
         </is>
       </c>
-      <c r="B94" s="9" t="n"/>
+      <c r="B94" s="7" t="n"/>
       <c r="C94" s="6" t="inlineStr">
         <is>
           <t>利用料</t>
@@ -1727,7 +1715,7 @@
           <t>特定事業所加算</t>
         </is>
       </c>
-      <c r="B95" s="9" t="n"/>
+      <c r="B95" s="7" t="n"/>
       <c r="C95" s="3" t="inlineStr">
         <is>
           <t>（Ⅰ）所定単位数の20/100
@@ -1754,7 +1742,7 @@
           <t>緊急時訪問介護加算</t>
         </is>
       </c>
-      <c r="B96" s="9" t="n"/>
+      <c r="B96" s="7" t="n"/>
       <c r="C96" s="3" t="inlineStr">
         <is>
           <t>1,112円</t>
@@ -1777,7 +1765,7 @@
           <t>初回加算</t>
         </is>
       </c>
-      <c r="B97" s="9" t="n"/>
+      <c r="B97" s="7" t="n"/>
       <c r="C97" s="3" t="inlineStr">
         <is>
           <t>2,224円</t>
@@ -1800,7 +1788,7 @@
           <t>中山間地域等における小規模事業所加算</t>
         </is>
       </c>
-      <c r="B98" s="9" t="n"/>
+      <c r="B98" s="7" t="n"/>
       <c r="C98" s="3" t="inlineStr">
         <is>
           <t>所定単位数の10/100</t>
@@ -1823,7 +1811,7 @@
           <t>中山間地域等に居住する者へのサービス提供加算</t>
         </is>
       </c>
-      <c r="B99" s="9" t="n"/>
+      <c r="B99" s="7" t="n"/>
       <c r="C99" s="3" t="inlineStr">
         <is>
           <t>所定単位数の5/100</t>
@@ -1847,7 +1835,7 @@
 生活機能向上連携加算(Ⅱ)</t>
         </is>
       </c>
-      <c r="B100" s="9" t="n"/>
+      <c r="B100" s="7" t="n"/>
       <c r="C100" s="3" t="inlineStr">
         <is>
           <t>(Ⅰ)1,112円
@@ -1873,7 +1861,7 @@
 訪問介護認知症専門ケア加算（Ⅱ）</t>
         </is>
       </c>
-      <c r="B101" s="9" t="n"/>
+      <c r="B101" s="7" t="n"/>
       <c r="C101" s="3" t="inlineStr">
         <is>
           <t>（Ⅰ）33円
@@ -1898,7 +1886,7 @@
           <t>口腔連携強化加算</t>
         </is>
       </c>
-      <c r="B102" s="9" t="n"/>
+      <c r="B102" s="7" t="n"/>
       <c r="C102" s="3" t="inlineStr">
         <is>
           <t>556円</t>
@@ -1922,7 +1910,7 @@
 （要介護度による区分なし）</t>
         </is>
       </c>
-      <c r="B103" s="9" t="n"/>
+      <c r="B103" s="7" t="n"/>
       <c r="C103" s="3" t="inlineStr">
         <is>
           <t>（Ⅰ）所定単位数の245/1000
@@ -2864,7 +2852,7 @@
 いいかいご事業部</t>
         </is>
       </c>
-      <c r="B230" s="9" t="n"/>
+      <c r="B230" s="7" t="n"/>
       <c r="C230" s="3" t="inlineStr">
         <is>
           <t>所在地　〒543-0023 大阪府大阪市天王寺区味原町13-18 オーセント味原302号室
@@ -2883,7 +2871,7 @@
 介護保険課</t>
         </is>
       </c>
-      <c r="B231" s="9" t="n"/>
+      <c r="B231" s="7" t="n"/>
       <c r="C231" s="3" t="inlineStr">
         <is>
           <t>所在地 大阪市中央区船場中央3-7-331
@@ -2904,7 +2892,7 @@
 （指定・指導グループ）</t>
         </is>
       </c>
-      <c r="B232" s="9" t="n"/>
+      <c r="B232" s="7" t="n"/>
       <c r="C232" s="3" t="inlineStr">
         <is>
           <t>大阪市中央区船場中央３丁目１番7-331
@@ -2922,7 +2910,7 @@
 大阪府国民健康保険団体連合会</t>
         </is>
       </c>
-      <c r="B233" s="9" t="n"/>
+      <c r="B233" s="7" t="n"/>
       <c r="C233" s="3" t="inlineStr">
         <is>
           <t>所在地 大阪市中央区常盤町1-3-8
@@ -3020,7 +3008,7 @@
       <c r="D246" s="4" t="n"/>
       <c r="E246" s="4" t="n"/>
     </row>
-    <row r="248" ht="18" customHeight="1">
+    <row r="248" ht="30" customHeight="1">
       <c r="A248" s="6" t="inlineStr">
         <is>
           <t>事業者</t>
@@ -3031,13 +3019,13 @@
           <t>所在地</t>
         </is>
       </c>
-      <c r="C248" s="7" t="inlineStr">
-        <is>
-          <t>【要入力】</t>
-        </is>
-      </c>
-      <c r="D248" s="8" t="n"/>
-      <c r="E248" s="8" t="n"/>
+      <c r="C248" s="3" t="inlineStr">
+        <is>
+          <t>〒541-0058 大阪府大阪市中央区南久宝寺町四丁目5番17号 アップウェル船場 2F</t>
+        </is>
+      </c>
+      <c r="D248" s="4" t="n"/>
+      <c r="E248" s="4" t="n"/>
     </row>
     <row r="249" ht="18" customHeight="1">
       <c r="A249" s="6" t="inlineStr">
@@ -3488,96 +3476,96 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>法人名</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>株式会社AA → 株式会社dhpケアマネジメント（ご指示どおり）</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>事業所名</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>ええかいご → いいかいご（ご指示どおり）</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>管理者・サービス提供責任者等</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>抜屋 壮勇 → 生田 友哉（ご指示どおり）</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>黄色セル</t>
-        </is>
-      </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>【要入力】：いいかいご／新法人の情報が手元にないため空欄。本社所在地・法人設立年月日・署名欄の事業者所在地</t>
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>要入力</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>なし（すべて入力済み）</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>コメント付きセル</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>旧事業所の内容をそのまま残した箇所（実施地域・損害賠償保険など）。要確認</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>説明年月日・利用者欄</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>新しく使えるよう空欄にしています</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>元の資料</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>重要事項説明書（訪問介護用）写真15ページ（重複1枚を除外）</t>
         </is>

</xml_diff>